<commit_message>
Use 'Jose' without accent; add one-page PDF summary
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KwpV9LZvKzSYSrQ38bwaGh
</commit_message>
<xml_diff>
--- a/Septiembre_2026_Horas_y_Kilometros.xlsx
+++ b/Septiembre_2026_Horas_y_Kilometros.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1 - Horas José y Emilio" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="1 - Horas Jose y Emilio" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2 - Tractor Saba Pistachio" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="3 - Km gasolina José y Emilio" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="3 - Km gasolina Jose y Emilio" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -558,23 +558,23 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>José y Emilio</t>
+          <t>Jose y Emilio</t>
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNT('1 - Horas José y Emilio'!A5:A22)</f>
+        <f>COUNT('1 - Horas Jose y Emilio'!A5:A22)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>'1 - Horas José y Emilio'!E23</f>
+        <f>'1 - Horas Jose y Emilio'!E23</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>'1 - Horas José y Emilio'!F23</f>
+        <f>'1 - Horas Jose y Emilio'!F23</f>
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>'3 - Km gasolina José y Emilio'!E10</f>
+        <f>'3 - Km gasolina Jose y Emilio'!E10</f>
         <v/>
       </c>
     </row>
@@ -618,7 +618,7 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Las horas totales de José y Emilio son personas × horas de cada día. La del tractor es una sola persona.</t>
+          <t>Las horas totales de Jose y Emilio son personas × horas de cada día. La del tractor es una sola persona.</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Horas trabajadas – José y Emilio</t>
+          <t>Horas trabajadas – Jose y Emilio</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Kilómetros de gasolina – José y Emilio</t>
+          <t>Kilómetros de gasolina – Jose y Emilio</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>TOTAL José y Emilio</t>
+          <t>TOTAL Jose y Emilio</t>
         </is>
       </c>
       <c r="B10" s="8">

</xml_diff>

<commit_message>
Add table 4: pistachio harvest hours per worker
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KwpV9LZvKzSYSrQ38bwaGh
</commit_message>
<xml_diff>
--- a/Septiembre_2026_Horas_y_Kilometros.xlsx
+++ b/Septiembre_2026_Horas_y_Kilometros.xlsx
@@ -11,6 +11,7 @@
     <sheet name="1 - Horas Jose y Emilio" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2 - Tractor Saba Pistachio" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="3 - Km gasolina Jose y Emilio" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="4 - Horas recogida pistachos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -60,7 +61,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +76,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,6 +137,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -565,11 +580,11 @@
         <f>COUNT('1 - Horas Jose y Emilio'!A5:A22)</f>
         <v/>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="15">
         <f>'1 - Horas Jose y Emilio'!E23</f>
         <v/>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="15">
         <f>'1 - Horas Jose y Emilio'!F23</f>
         <v/>
       </c>
@@ -588,11 +603,11 @@
         <f>COUNT('2 - Tractor Saba Pistachio'!C5:C11)</f>
         <v/>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="15">
         <f>'2 - Tractor Saba Pistachio'!C12</f>
         <v/>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="15">
         <f>C6</f>
         <v/>
       </c>
@@ -706,10 +721,10 @@
       <c r="D5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="15">
         <f>D5*E5</f>
         <v/>
       </c>
@@ -729,10 +744,10 @@
       <c r="D6" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="15">
         <f>D6*E6</f>
         <v/>
       </c>
@@ -752,10 +767,10 @@
       <c r="D7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="15">
         <f>D7*E7</f>
         <v/>
       </c>
@@ -775,10 +790,10 @@
       <c r="D8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="15" t="n">
         <v>7.5</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="15">
         <f>D8*E8</f>
         <v/>
       </c>
@@ -798,10 +813,10 @@
       <c r="D9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="15">
         <f>D9*E9</f>
         <v/>
       </c>
@@ -821,10 +836,10 @@
       <c r="D10" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="15">
         <f>D10*E10</f>
         <v/>
       </c>
@@ -844,10 +859,10 @@
       <c r="D11" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="15">
         <f>D11*E11</f>
         <v/>
       </c>
@@ -867,10 +882,10 @@
       <c r="D12" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="15">
         <f>D12*E12</f>
         <v/>
       </c>
@@ -890,10 +905,10 @@
       <c r="D13" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="15">
         <f>D13*E13</f>
         <v/>
       </c>
@@ -913,10 +928,10 @@
       <c r="D14" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="15">
         <f>D14*E14</f>
         <v/>
       </c>
@@ -936,10 +951,10 @@
       <c r="D15" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="15">
         <f>D15*E15</f>
         <v/>
       </c>
@@ -959,10 +974,10 @@
       <c r="D16" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="15" t="n">
         <v>6.5</v>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="15">
         <f>D16*E16</f>
         <v/>
       </c>
@@ -982,10 +997,10 @@
       <c r="D17" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="15">
         <f>D17*E17</f>
         <v/>
       </c>
@@ -1005,10 +1020,10 @@
       <c r="D18" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="15" t="n">
         <v>9.5</v>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="15">
         <f>D18*E18</f>
         <v/>
       </c>
@@ -1028,10 +1043,10 @@
       <c r="D19" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="15">
         <f>D19*E19</f>
         <v/>
       </c>
@@ -1051,10 +1066,10 @@
       <c r="D20" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="15" t="n">
         <v>10.5</v>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="15">
         <f>D20*E20</f>
         <v/>
       </c>
@@ -1074,10 +1089,10 @@
       <c r="D21" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="E21" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="F21" s="12">
+      <c r="F21" s="15">
         <f>D21*E21</f>
         <v/>
       </c>
@@ -1097,10 +1112,10 @@
       <c r="D22" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E22" s="12" t="n">
+      <c r="E22" s="15" t="n">
         <v>1.5</v>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="15">
         <f>D22*E22</f>
         <v/>
       </c>
@@ -1117,11 +1132,11 @@
       </c>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
-      <c r="E23" s="13">
+      <c r="E23" s="16">
         <f>SUM(E5:E22)</f>
         <v/>
       </c>
-      <c r="F23" s="13">
+      <c r="F23" s="16">
         <f>SUM(F5:F22)</f>
         <v/>
       </c>
@@ -1199,7 +1214,7 @@
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="15" t="n">
         <v>10.5</v>
       </c>
       <c r="D5" s="5" t="n">
@@ -1215,7 +1230,7 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="15" t="n">
         <v>12</v>
       </c>
       <c r="D6" s="5" t="n">
@@ -1231,7 +1246,7 @@
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="15" t="n">
         <v>12</v>
       </c>
       <c r="D7" s="5" t="n">
@@ -1247,7 +1262,7 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="15" t="n">
         <v>12</v>
       </c>
       <c r="D8" s="5" t="n">
@@ -1263,7 +1278,7 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="15" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="5" t="n">
@@ -1279,7 +1294,7 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="15" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="5" t="n">
@@ -1295,7 +1310,7 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="15" t="n">
         <v>12</v>
       </c>
       <c r="D11" s="5" t="n">
@@ -1312,7 +1327,7 @@
         <f>COUNT(C5:C11)&amp;" días"</f>
         <v/>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="16">
         <f>SUM(C5:C11)</f>
         <v/>
       </c>
@@ -1517,4 +1532,394 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Horas por trabajador – recogida de pistachos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Septiembre 2026 · Datos copiados de una nota escrita a mano · Celdas amarillas = pendientes de confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Trabajador</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Horas (sin desglosar)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Horas Jose</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Horas Máquina</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Horas Saba</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Total horas</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Lois</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5">
+        <f>SUM(B5:E5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Nombre dudoso (¿Luis?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Beto</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5">
+        <f>SUM(B6:E6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="13" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Leiner</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5">
+        <f>SUM(B7:E7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Número dudoso: ¿45 o 46?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>266</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="F8" s="5">
+        <f>SUM(B8:E8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>En la nota el total escrito es 315</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Marck</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5">
+        <f>SUM(B9:E9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Alberto</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5">
+        <f>SUM(B10:E10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Loimar</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5">
+        <f>SUM(B11:E11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="13" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Jair</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5">
+        <f>SUM(B12:E12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="13" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Henry</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5">
+        <f>SUM(B13:E13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Ruben</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5">
+        <f>SUM(B14:E14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="13" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Elis</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5">
+        <f>SUM(B15:E15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="13" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sebastian</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5">
+        <f>SUM(B16:E16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="13" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Isidro</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5">
+        <f>SUM(B17:E17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>Tras el 25 hay texto ilegible y «2 días»; pendiente de confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Braian</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>29</v>
+      </c>
+      <c r="F18" s="5">
+        <f>SUM(B18:E18)</f>
+        <v/>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>Reparto Jose/Máquina/Saba leído por analogía con Jorge; pendiente de confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B19" s="8">
+        <f>SUM(B5:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="8">
+        <f>SUM(C5:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="8">
+        <f>SUM(D5:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="8">
+        <f>SUM(E5:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="8">
+        <f>SUM(F5:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Las horas «Jose», «Máquina» y «Saba» indican para quién o con qué se trabajaron. Las demás líneas no indicaban desglose.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update table 4 with confirmed names and Bryan hours
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KwpV9LZvKzSYSrQ38bwaGh
</commit_message>
<xml_diff>
--- a/Septiembre_2026_Horas_y_Kilometros.xlsx
+++ b/Septiembre_2026_Horas_y_Kilometros.xlsx
@@ -110,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,9 +138,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
@@ -580,11 +577,11 @@
         <f>COUNT('1 - Horas Jose y Emilio'!A5:A22)</f>
         <v/>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="14">
         <f>'1 - Horas Jose y Emilio'!E23</f>
         <v/>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="14">
         <f>'1 - Horas Jose y Emilio'!F23</f>
         <v/>
       </c>
@@ -603,11 +600,11 @@
         <f>COUNT('2 - Tractor Saba Pistachio'!C5:C11)</f>
         <v/>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="14">
         <f>'2 - Tractor Saba Pistachio'!C12</f>
         <v/>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="14">
         <f>C6</f>
         <v/>
       </c>
@@ -721,10 +718,10 @@
       <c r="D5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="14">
         <f>D5*E5</f>
         <v/>
       </c>
@@ -744,10 +741,10 @@
       <c r="D6" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="14">
         <f>D6*E6</f>
         <v/>
       </c>
@@ -767,10 +764,10 @@
       <c r="D7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="14">
         <f>D7*E7</f>
         <v/>
       </c>
@@ -790,10 +787,10 @@
       <c r="D8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="14" t="n">
         <v>7.5</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="14">
         <f>D8*E8</f>
         <v/>
       </c>
@@ -813,10 +810,10 @@
       <c r="D9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="14">
         <f>D9*E9</f>
         <v/>
       </c>
@@ -836,10 +833,10 @@
       <c r="D10" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="14">
         <f>D10*E10</f>
         <v/>
       </c>
@@ -859,10 +856,10 @@
       <c r="D11" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="14">
         <f>D11*E11</f>
         <v/>
       </c>
@@ -882,10 +879,10 @@
       <c r="D12" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="14">
         <f>D12*E12</f>
         <v/>
       </c>
@@ -905,10 +902,10 @@
       <c r="D13" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="14">
         <f>D13*E13</f>
         <v/>
       </c>
@@ -928,10 +925,10 @@
       <c r="D14" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="14">
         <f>D14*E14</f>
         <v/>
       </c>
@@ -951,10 +948,10 @@
       <c r="D15" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="14">
         <f>D15*E15</f>
         <v/>
       </c>
@@ -974,10 +971,10 @@
       <c r="D16" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="E16" s="14" t="n">
         <v>6.5</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="14">
         <f>D16*E16</f>
         <v/>
       </c>
@@ -997,10 +994,10 @@
       <c r="D17" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="14">
         <f>D17*E17</f>
         <v/>
       </c>
@@ -1020,10 +1017,10 @@
       <c r="D18" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="E18" s="14" t="n">
         <v>9.5</v>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="14">
         <f>D18*E18</f>
         <v/>
       </c>
@@ -1043,10 +1040,10 @@
       <c r="D19" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="E19" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="14">
         <f>D19*E19</f>
         <v/>
       </c>
@@ -1066,10 +1063,10 @@
       <c r="D20" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E20" s="15" t="n">
+      <c r="E20" s="14" t="n">
         <v>10.5</v>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="14">
         <f>D20*E20</f>
         <v/>
       </c>
@@ -1089,10 +1086,10 @@
       <c r="D21" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="E21" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="F21" s="15">
+      <c r="F21" s="14">
         <f>D21*E21</f>
         <v/>
       </c>
@@ -1112,10 +1109,10 @@
       <c r="D22" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E22" s="15" t="n">
+      <c r="E22" s="14" t="n">
         <v>1.5</v>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="14">
         <f>D22*E22</f>
         <v/>
       </c>
@@ -1132,11 +1129,11 @@
       </c>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
-      <c r="E23" s="16">
+      <c r="E23" s="15">
         <f>SUM(E5:E22)</f>
         <v/>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="15">
         <f>SUM(F5:F22)</f>
         <v/>
       </c>
@@ -1214,7 +1211,7 @@
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="14" t="n">
         <v>10.5</v>
       </c>
       <c r="D5" s="5" t="n">
@@ -1230,7 +1227,7 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="14" t="n">
         <v>12</v>
       </c>
       <c r="D6" s="5" t="n">
@@ -1246,7 +1243,7 @@
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="14" t="n">
         <v>12</v>
       </c>
       <c r="D7" s="5" t="n">
@@ -1262,7 +1259,7 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="14" t="n">
         <v>12</v>
       </c>
       <c r="D8" s="5" t="n">
@@ -1278,7 +1275,7 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="14" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="5" t="n">
@@ -1294,7 +1291,7 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="14" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="5" t="n">
@@ -1310,7 +1307,7 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="14" t="n">
         <v>12</v>
       </c>
       <c r="D11" s="5" t="n">
@@ -1327,7 +1324,7 @@
         <f>COUNT(C5:C11)&amp;" días"</f>
         <v/>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="15">
         <f>SUM(C5:C11)</f>
         <v/>
       </c>
@@ -1604,7 +1601,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Lois</t>
         </is>
@@ -1619,11 +1616,7 @@
         <f>SUM(B5:E5)</f>
         <v/>
       </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>Nombre dudoso (¿Luis?)</t>
-        </is>
-      </c>
+      <c r="G5" s="12" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1641,7 +1634,7 @@
         <f>SUM(B6:E6)</f>
         <v/>
       </c>
-      <c r="G6" s="13" t="inlineStr"/>
+      <c r="G6" s="12" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1649,7 +1642,7 @@
           <t>Leiner</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="5" t="n">
         <v>46</v>
       </c>
       <c r="C7" s="5" t="n"/>
@@ -1659,11 +1652,7 @@
         <f>SUM(B7:E7)</f>
         <v/>
       </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>Número dudoso: ¿45 o 46?</t>
-        </is>
-      </c>
+      <c r="G7" s="12" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1685,7 +1674,7 @@
         <f>SUM(B8:E8)</f>
         <v/>
       </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>En la nota el total escrito es 315</t>
         </is>
@@ -1707,7 +1696,7 @@
         <f>SUM(B9:E9)</f>
         <v/>
       </c>
-      <c r="G9" s="13" t="inlineStr"/>
+      <c r="G9" s="12" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1725,7 +1714,7 @@
         <f>SUM(B10:E10)</f>
         <v/>
       </c>
-      <c r="G10" s="13" t="inlineStr"/>
+      <c r="G10" s="12" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1743,7 +1732,7 @@
         <f>SUM(B11:E11)</f>
         <v/>
       </c>
-      <c r="G11" s="13" t="inlineStr"/>
+      <c r="G11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1761,12 +1750,12 @@
         <f>SUM(B12:E12)</f>
         <v/>
       </c>
-      <c r="G12" s="13" t="inlineStr"/>
+      <c r="G12" s="12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Henry</t>
+          <t>Jenrry</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -1779,7 +1768,7 @@
         <f>SUM(B13:E13)</f>
         <v/>
       </c>
-      <c r="G13" s="13" t="inlineStr"/>
+      <c r="G13" s="12" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1797,7 +1786,7 @@
         <f>SUM(B14:E14)</f>
         <v/>
       </c>
-      <c r="G14" s="13" t="inlineStr"/>
+      <c r="G14" s="12" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1815,7 +1804,7 @@
         <f>SUM(B15:E15)</f>
         <v/>
       </c>
-      <c r="G15" s="13" t="inlineStr"/>
+      <c r="G15" s="12" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1833,7 +1822,7 @@
         <f>SUM(B16:E16)</f>
         <v/>
       </c>
-      <c r="G16" s="13" t="inlineStr"/>
+      <c r="G16" s="12" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1841,7 +1830,7 @@
           <t>Isidro</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B17" s="13" t="n">
         <v>25</v>
       </c>
       <c r="C17" s="5" t="n"/>
@@ -1851,7 +1840,7 @@
         <f>SUM(B17:E17)</f>
         <v/>
       </c>
-      <c r="G17" s="13" t="inlineStr">
+      <c r="G17" s="12" t="inlineStr">
         <is>
           <t>Tras el 25 hay texto ilegible y «2 días»; pendiente de confirmar</t>
         </is>
@@ -1860,28 +1849,24 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Braian</t>
+          <t>Bryan</t>
         </is>
       </c>
       <c r="B18" s="5" t="n"/>
-      <c r="C18" s="14" t="n">
+      <c r="C18" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="D18" s="14" t="n">
-        <v>30</v>
-      </c>
-      <c r="E18" s="14" t="n">
+      <c r="D18" s="5" t="n">
+        <v>304</v>
+      </c>
+      <c r="E18" s="5" t="n">
         <v>29</v>
       </c>
       <c r="F18" s="5">
         <f>SUM(B18:E18)</f>
         <v/>
       </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>Reparto Jose/Máquina/Saba leído por analogía con Jorge; pendiente de confirmar</t>
-        </is>
-      </c>
+      <c r="G18" s="12" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">

</xml_diff>